<commit_message>
feat: enrich sample Excel data and regenerate UI mock JSON
Expand the fictional demo dataset and wire mock-data generation through
the real validation/allocation/aging/export pipeline so the static UI
reflects realistic multi-row results instead of single-row fixtures.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/sample_data/sample_inventory.xlsx
+++ b/sample_data/sample_inventory.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,7 +456,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MED-LENS-001</t>
+          <t>VIS-SLIT-001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -465,56 +465,56 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Vista Optics Supply</t>
+          <t>Reingold Optical Instruments Ltd</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>18</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MED-LENS-001</t>
+          <t>VIS-SLIT-001</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SG Warehouse</t>
+          <t>Europe Warehouse</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Vista Optics Supply</t>
+          <t>Reingold Optical Instruments Ltd</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>MED-GLOVE-002</t>
+          <t>VIS-LENS-002</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -523,46 +523,46 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E4" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Everclean Medical Supply</t>
+          <t>Pearl Vision Manufacturing Ltd</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MED-GLOVE-002</t>
+          <t>VIS-LENS-002</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SG Warehouse</t>
+          <t>China Warehouse</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="D5" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Everclean Medical Supply</t>
+          <t>Pearl Vision Manufacturing Ltd</t>
         </is>
       </c>
       <c r="G5" t="n">
@@ -572,7 +572,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MED-MASK-003</t>
+          <t>VIS-REFR-003</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -581,27 +581,27 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>100</v>
+        <v>6</v>
       </c>
       <c r="D6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Everclean Medical Supply</t>
+          <t>Reingold Optical Instruments Ltd</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>IND-VALVE-004</t>
+          <t>DIAG-OCT-005</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -610,56 +610,56 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Precision Hydraulics Ltd</t>
+          <t>Meridian Diagnostics Co</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>21</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>IND-VALVE-004</t>
+          <t>DIAG-OCT-005</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>SG Warehouse</t>
+          <t>Europe Warehouse</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8" t="n">
         <v>2</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Precision Hydraulics Ltd</t>
+          <t>Meridian Diagnostics Co</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>21</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>IND-PUMP-005</t>
+          <t>DIAG-FUND-006</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -668,27 +668,27 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Precision Hydraulics Ltd</t>
+          <t>Meridian Diagnostics Co</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>OFF-CHAIR-006</t>
+          <t>DIAG-TONO-007</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -697,50 +697,253 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Comfort Seating Supply Co</t>
+          <t>Meridian Diagnostics Co</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>30</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>OFF-DESK-007</t>
+          <t>DIAG-TONO-007</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>SG Warehouse</t>
+          <t>China Warehouse</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D11" t="n">
         <v>2</v>
       </c>
       <c r="E11" t="n">
+        <v>4</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Meridian Diagnostics Co</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>DIAG-AUTO-008</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>China Warehouse</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>12</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>4</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Meridian Diagnostics Co</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>CONS-WIPE-009</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>HK Warehouse</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>300</v>
+      </c>
+      <c r="D13" t="n">
+        <v>20</v>
+      </c>
+      <c r="E13" t="n">
+        <v>50</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Everclean Medical Supply</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CONS-DROP-010</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>HK Warehouse</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>150</v>
+      </c>
+      <c r="D14" t="n">
+        <v>10</v>
+      </c>
+      <c r="E14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Everclean Medical Supply</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>CONS-COVER-011</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>China Warehouse</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>400</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>60</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Everclean Medical Supply</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
         <v>5</v>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Comfort Seating Supply Co</t>
-        </is>
-      </c>
-      <c r="G11" t="n">
-        <v>30</v>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>CONS-CALSTRIP-012</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>HK Warehouse</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>90</v>
+      </c>
+      <c r="D16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E16" t="n">
+        <v>20</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Meridian Diagnostics Co</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>PART-BULB-013</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>HK Warehouse</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>25</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>8</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Reingold Optical Instruments Ltd</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>PART-CHINREST-014</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>China Warehouse</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>18</v>
+      </c>
+      <c r="D18" t="n">
+        <v>2</v>
+      </c>
+      <c r="E18" t="n">
+        <v>6</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Pearl Vision Manufacturing Ltd</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>